<commit_message>
Add consistent cell borders to assessment Excel exports
</commit_message>
<xml_diff>
--- a/assets/assessment/control-template.xlsx
+++ b/assets/assessment/control-template.xlsx
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -98,45 +98,60 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8BEC7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8BEC7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB8BEC7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB8BEC7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -179,6 +194,41 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30">
       <c r="A3" s="5" t="inlineStr">
@@ -191,6 +241,41 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30">
       <c r="A4" s="5" t="inlineStr">
@@ -203,6 +288,41 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30">
       <c r="A5" s="5" t="inlineStr">
@@ -215,6 +335,41 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30">
       <c r="A6" s="5" t="inlineStr">
@@ -223,6 +378,41 @@
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>